<commit_message>
Record 2026-04-28 job post count
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$2</c:f>
+              <c:f>Data!$A$2:$A$3</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$2</c:f>
+              <c:f>Data!$C$2:$C$3</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -398,8 +398,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-28 23:47:45</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>200182</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>parsed joblist hdnGICnt</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F2"/>
+  <autoFilter ref="A1:F3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -456,13 +486,13 @@
         <v>186993</v>
       </c>
       <c r="C2">
-        <v>186993</v>
+        <v>200182</v>
       </c>
       <c r="D2">
         <v>186993</v>
       </c>
       <c r="E2">
-        <v>186993</v>
+        <v>200182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update job post counts
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$3</c:f>
+              <c:f>Data!$A$2:$A$4</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$3</c:f>
+              <c:f>Data!$C$2:$C$4</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -428,8 +428,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-29 12:38:49</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>199111</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>parsed joblist hdnGICnt</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
+  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -492,7 +522,7 @@
         <v>186993</v>
       </c>
       <c r="E2">
-        <v>200182</v>
+        <v>199111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exclude failed measurements from candle charts
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$5</c:f>
+              <c:f>Data!$A$2:$A$4</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$5</c:f>
+              <c:f>Data!$C$2:$C$4</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -458,40 +458,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-04-29 14:08:00</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>WinHttpSendRequest failed.</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F4"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Keep one daily job count record
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$9</c:f>
+              <c:f>Data!$A$2:$A$5</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$9</c:f>
+              <c:f>Data!$C$2:$C$5</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -488,128 +488,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-04-30 12:22:26</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>199915</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>parsed joblist hdnGICnt</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-04-30 12:28:08</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C7">
-        <v>199967</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>parsed joblist hdnGICnt</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-04-30 12:30:10</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>199967</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>parsed joblist hdnGICnt</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-04-30 12:33:51</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>199984</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>parsed joblist hdnGICnt</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -672,7 +552,7 @@
         <v>186993</v>
       </c>
       <c r="E2">
-        <v>199984</v>
+        <v>197667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manually update June 5 job count
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -1541,7 +1541,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-05 09:00:55</t>
+          <t>2026-06-05 09:46:39</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1549,19 +1549,17 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="C41">
+        <v>194086</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>ok</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>HTTP failed after 3 attempts: WinHttpSendRequest failed.</t>
+          <t>parsed joblist hdnGICnt</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1723,13 +1721,13 @@
         <v>180449</v>
       </c>
       <c r="C7">
-        <v>190777</v>
+        <v>194086</v>
       </c>
       <c r="D7">
         <v>180449</v>
       </c>
       <c r="E7">
-        <v>187906</v>
+        <v>194086</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Record external JobKorea count
</commit_message>
<xml_diff>
--- a/data/job_post_counts.xlsx
+++ b/data/job_post_counts.xlsx
@@ -81,12 +81,12 @@
           </c:tx>
           <c:cat>
             <c:strRef>
-              <c:f>Data!$A$2:$A$41</c:f>
+              <c:f>Data!$A$2:$A$42</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Data!$C$2:$C$41</c:f>
+              <c:f>Data!$C$2:$C$42</c:f>
             </c:numRef>
           </c:val>
         </c:ser>
@@ -1568,8 +1568,38 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-06-06 09:00:36</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="C42">
+        <v>193724</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>parsed joblist hdnGICnt</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.jobkorea.co.kr/recruit/joblist?menucode=local&amp;localorder=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F41"/>
+  <autoFilter ref="A1:F42"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1727,7 +1757,7 @@
         <v>180449</v>
       </c>
       <c r="E7">
-        <v>194086</v>
+        <v>193724</v>
       </c>
     </row>
   </sheetData>

</xml_diff>